<commit_message>
Added more test cases (#838)
</commit_message>
<xml_diff>
--- a/php-zigar/tests/test-matrix.xlsx
+++ b/php-zigar/tests/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1769884350" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1769884350" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1769884350" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1769884350"/>
+      <pm:revision xmlns:pm="smNativeData" day="1769902809" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1769902809" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1769902809" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1769902809"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="106">
   <si>
     <t>Context</t>
   </si>
@@ -115,6 +115,9 @@
     <t>As static variable</t>
   </si>
   <si>
+    <t>N</t>
+  </si>
+  <si>
     <t>Y</t>
   </si>
   <si>
@@ -149,9 +152,6 @@
   </si>
   <si>
     <t>Vector of</t>
-  </si>
-  <si>
-    <t>N</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -382,7 +382,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769884350" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769902809" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -397,7 +397,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769884350" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769902809" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -412,7 +412,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769884350" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769902809" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -428,7 +428,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769884350" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769902809" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -450,7 +450,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -461,7 +461,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -472,7 +472,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -483,7 +483,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -494,7 +494,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -505,7 +505,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769884350" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -527,7 +527,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350"/>
+          <pm:border xmlns:pm="smNativeData" id="1769902809"/>
         </ext>
       </extLst>
     </border>
@@ -546,7 +546,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350">
+          <pm:border xmlns:pm="smNativeData" id="1769902809">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -568,7 +568,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350">
+          <pm:border xmlns:pm="smNativeData" id="1769902809">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -592,7 +592,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350">
+          <pm:border xmlns:pm="smNativeData" id="1769902809">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -616,7 +616,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350">
+          <pm:border xmlns:pm="smNativeData" id="1769902809">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -640,7 +640,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350"/>
+          <pm:border xmlns:pm="smNativeData" id="1769902809"/>
         </ext>
       </extLst>
     </border>
@@ -659,7 +659,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769884350"/>
+          <pm:border xmlns:pm="smNativeData" id="1769902809"/>
         </ext>
       </extLst>
     </border>
@@ -709,13 +709,87 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769902809" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769902809" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769902809" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769902809" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1769884350" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1769902809" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1769884350" count="5">
+      <pm:colors xmlns:pm="smNativeData" id="1769902809" count="5">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1124,12 +1198,16 @@
         <v>25</v>
       </c>
       <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
+      <c r="C3" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="D3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="F3" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
@@ -1152,15 +1230,19 @@
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
       <c r="D4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
@@ -1183,15 +1265,19 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
+      <c r="C5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="D5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
@@ -1214,15 +1300,19 @@
     </row>
     <row r="6" spans="1:25">
       <c r="A6" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
+      <c r="C6" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="D6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
@@ -1245,7 +1335,7 @@
     </row>
     <row r="7" spans="1:25">
       <c r="A7" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1274,7 +1364,7 @@
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1303,7 +1393,7 @@
     </row>
     <row r="9" spans="1:25">
       <c r="A9" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1332,7 +1422,7 @@
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -1361,7 +1451,7 @@
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1390,15 +1480,19 @@
     </row>
     <row r="12" spans="1:25">
       <c r="A12" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
+      <c r="C12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="D12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
+      <c r="F12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
@@ -1421,7 +1515,7 @@
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1450,15 +1544,19 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
+      <c r="C14" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="D14" s="10" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
@@ -1484,10 +1582,25 @@
     <mergeCell ref="B1:Y1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:Y14">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C14">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:Y14">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1496,14 +1609,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1562,7 +1675,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1573,14 +1686,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1631,7 +1744,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1642,14 +1755,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1738,7 +1851,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1749,14 +1862,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1809,7 +1922,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1820,14 +1933,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1874,7 +1987,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1885,14 +1998,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1965,7 +2078,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1976,14 +2089,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2022,7 +2135,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2033,14 +2146,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2201,7 +2314,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2212,14 +2325,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2290,7 +2403,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2301,14 +2414,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2367,7 +2480,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2378,14 +2491,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2456,7 +2569,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2467,14 +2580,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2539,7 +2652,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769884350" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769902809" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2550,14 +2663,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769884350" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769902809" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769884350" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769902809" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Copied more tests from zigar-compiler (#838)
</commit_message>
<xml_diff>
--- a/php-zigar/tests/test-matrix.xlsx
+++ b/php-zigar/tests/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1769916202" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1769916202" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1769916202" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1769916202"/>
+      <pm:revision xmlns:pm="smNativeData" day="1769990795" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1769990795" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1769990795" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1769990795"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="106">
   <si>
     <t>Context</t>
   </si>
@@ -382,7 +382,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769916202" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -397,7 +397,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769916202" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -412,7 +412,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769916202" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -428,7 +428,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769916202" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -437,7 +437,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -450,7 +450,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -461,7 +461,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -472,7 +472,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -483,7 +483,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -494,7 +494,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -505,13 +505,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -527,7 +538,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202"/>
+          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
         </ext>
       </extLst>
     </border>
@@ -546,7 +557,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202">
+          <pm:border xmlns:pm="smNativeData" id="1769990795">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -568,7 +579,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202">
+          <pm:border xmlns:pm="smNativeData" id="1769990795">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -592,7 +603,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202">
+          <pm:border xmlns:pm="smNativeData" id="1769990795">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -616,7 +627,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202">
+          <pm:border xmlns:pm="smNativeData" id="1769990795">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -640,7 +651,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202"/>
+          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
         </ext>
       </extLst>
     </border>
@@ -659,7 +670,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769916202"/>
+          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
         </ext>
       </extLst>
     </border>
@@ -709,13 +739,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="13">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769916202" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -728,7 +758,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -739,7 +769,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769916202" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -752,7 +782,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -763,7 +793,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769916202" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -776,7 +806,247 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769916202" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -786,10 +1056,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1769916202" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1769990795" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1769916202" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1769990795" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1217,15 +1487,21 @@
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
+      <c r="K3" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L3" s="10" t="s">
         <v>27</v>
       </c>
       <c r="M3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
+      <c r="N3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="P3" s="10"/>
       <c r="Q3" s="10"/>
       <c r="R3" s="10"/>
@@ -1235,7 +1511,9 @@
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
       <c r="X3" s="10"/>
-      <c r="Y3" s="10"/>
+      <c r="Y3" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="9" t="s">
@@ -1260,15 +1538,19 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
+      <c r="K4" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
       <c r="R4" s="10"/>
@@ -1278,7 +1560,9 @@
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
       <c r="X4" s="10"/>
-      <c r="Y4" s="10"/>
+      <c r="Y4" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="9" t="s">
@@ -1303,15 +1587,19 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
+      <c r="K5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
       <c r="R5" s="10"/>
@@ -1321,7 +1609,9 @@
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="10"/>
-      <c r="Y5" s="10"/>
+      <c r="Y5" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" s="9" t="s">
@@ -1349,8 +1639,12 @@
         <v>26</v>
       </c>
       <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
+      <c r="N6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
       <c r="R6" s="10"/>
@@ -1391,7 +1685,9 @@
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
       <c r="X7" s="10"/>
-      <c r="Y7" s="10"/>
+      <c r="Y7" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="9" t="s">
@@ -1408,15 +1704,21 @@
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
+      <c r="K8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L8" s="10" t="s">
         <v>27</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
+      <c r="N8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="10"/>
       <c r="R8" s="10"/>
@@ -1426,7 +1728,9 @@
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
       <c r="X8" s="10"/>
-      <c r="Y8" s="10"/>
+      <c r="Y8" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" s="9" t="s">
@@ -1477,7 +1781,9 @@
       <c r="K10" s="10"/>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="N10" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
@@ -1544,14 +1850,16 @@
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
+      <c r="K12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="O12" s="10"/>
       <c r="P12" s="10"/>
       <c r="Q12" s="10"/>
@@ -1562,7 +1870,9 @@
       <c r="V12" s="11"/>
       <c r="W12" s="11"/>
       <c r="X12" s="10"/>
-      <c r="Y12" s="10"/>
+      <c r="Y12" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="9" t="s">
@@ -1574,7 +1884,9 @@
       <c r="E13" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="10"/>
+      <c r="F13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
@@ -1582,7 +1894,9 @@
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="N13" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
@@ -1593,7 +1907,9 @@
       <c r="V13" s="11"/>
       <c r="W13" s="11"/>
       <c r="X13" s="10"/>
-      <c r="Y13" s="10"/>
+      <c r="Y13" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="14" spans="1:25">
       <c r="A14" s="9" t="s">
@@ -1616,15 +1932,21 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
+      <c r="K14" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L14" s="10" t="s">
         <v>27</v>
       </c>
       <c r="M14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
+      <c r="N14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="10"/>
       <c r="R14" s="10"/>
@@ -1633,8 +1955,12 @@
       <c r="U14" s="10"/>
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
-      <c r="X14" s="10"/>
-      <c r="Y14" s="10"/>
+      <c r="X14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1659,7 +1985,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1668,14 +1994,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1734,7 +2060,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1745,14 +2071,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1803,7 +2129,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1814,14 +2140,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1910,7 +2236,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1921,14 +2247,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -1981,7 +2307,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1992,14 +2318,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2010,7 +2336,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="29.098214" customWidth="1" style="0"/>
@@ -2042,15 +2368,48 @@
         <v>27</v>
       </c>
     </row>
+    <row r="6" spans="2:2">
+      <c r="B6" s="10"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2061,14 +2420,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2141,7 +2500,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2152,14 +2511,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2198,7 +2557,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2209,14 +2568,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2227,7 +2586,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="35.062500" customWidth="1" style="0"/>
@@ -2247,13 +2606,17 @@
       <c r="A3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
@@ -2363,21 +2726,42 @@
       </c>
       <c r="B22" s="10"/>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
         <v>69</v>
       </c>
       <c r="B23" s="10"/>
+      <c r="D23" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
+  <conditionalFormatting sqref="D23">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B23">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B23">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2388,14 +2772,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2466,7 +2850,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2477,14 +2861,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2543,7 +2927,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2554,14 +2938,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2632,7 +3016,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2643,14 +3027,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2715,7 +3099,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769916202" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2726,14 +3110,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769916202" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769916202" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Finished tests for float
</commit_message>
<xml_diff>
--- a/php-zigar/tests/test-matrix.xlsx
+++ b/php-zigar/tests/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1769990795" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1769990795" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1769990795" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1769990795"/>
+      <pm:revision xmlns:pm="smNativeData" day="1772143101" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1772143101" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1772143101" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1772143101"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="107">
   <si>
     <t>Context</t>
   </si>
@@ -115,12 +115,12 @@
     <t>As static variable</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>As function parameters</t>
   </si>
   <si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Vector of</t>
+  </si>
+  <si>
+    <t>Constructor</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -382,7 +385,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -397,7 +400,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -412,7 +415,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -428,7 +431,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1769990795" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -450,7 +453,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -461,7 +464,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -472,7 +475,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -483,7 +486,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -494,7 +497,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -505,7 +508,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -516,7 +519,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -538,7 +541,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
+          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
         </ext>
       </extLst>
     </border>
@@ -557,7 +560,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795">
+          <pm:border xmlns:pm="smNativeData" id="1772143101">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -579,7 +582,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795">
+          <pm:border xmlns:pm="smNativeData" id="1772143101">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -603,7 +606,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795">
+          <pm:border xmlns:pm="smNativeData" id="1772143101">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -627,7 +630,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795">
+          <pm:border xmlns:pm="smNativeData" id="1772143101">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -651,7 +654,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
+          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
         </ext>
       </extLst>
     </border>
@@ -670,7 +673,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
+          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
         </ext>
       </extLst>
     </border>
@@ -689,7 +692,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1769990795"/>
+          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
         </ext>
       </extLst>
     </border>
@@ -739,13 +742,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="19">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -758,7 +761,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -769,7 +772,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -782,7 +785,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -793,7 +796,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -806,7 +809,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -817,7 +820,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -830,7 +833,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -841,7 +844,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -854,7 +857,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -865,7 +868,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -878,7 +881,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -889,7 +892,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -902,7 +905,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -913,7 +916,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -926,7 +929,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -937,7 +940,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -950,7 +953,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -961,7 +964,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -974,7 +977,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -985,7 +988,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -998,7 +1001,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1009,7 +1012,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1022,7 +1025,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1033,7 +1036,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1769990795" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1046,7 +1049,151 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1769990795" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1056,10 +1203,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1769990795" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1772143101" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1769990795" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1772143101" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1328,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="7" defaultColWidth="8.544643" defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="22.151786" customWidth="1" style="0"/>
@@ -1473,13 +1620,13 @@
         <v>26</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>26</v>
@@ -1488,19 +1635,19 @@
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
       <c r="K3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O3" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="M3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="O3" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="P3" s="10"/>
       <c r="Q3" s="10"/>
@@ -1512,7 +1659,7 @@
       <c r="W3" s="11"/>
       <c r="X3" s="10"/>
       <c r="Y3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1521,35 +1668,35 @@
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
       <c r="K4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
@@ -1561,7 +1708,7 @@
       <c r="W4" s="11"/>
       <c r="X4" s="10"/>
       <c r="Y4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1570,35 +1717,35 @@
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="F5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
       <c r="K5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M5" s="10"/>
       <c r="N5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
@@ -1610,7 +1757,7 @@
       <c r="W5" s="11"/>
       <c r="X5" s="10"/>
       <c r="Y5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1622,28 +1769,30 @@
         <v>26</v>
       </c>
       <c r="D6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="10"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
       <c r="L6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
@@ -1661,13 +1810,21 @@
         <v>31</v>
       </c>
       <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="C7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
@@ -1686,7 +1843,7 @@
       <c r="W7" s="11"/>
       <c r="X7" s="10"/>
       <c r="Y7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1694,30 +1851,38 @@
         <v>32</v>
       </c>
       <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="C8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="10"/>
@@ -1729,7 +1894,7 @@
       <c r="W8" s="11"/>
       <c r="X8" s="10"/>
       <c r="Y8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1737,13 +1902,21 @@
         <v>33</v>
       </c>
       <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="C9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E9" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
@@ -1768,13 +1941,21 @@
         <v>34</v>
       </c>
       <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
+      <c r="C10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E10" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
@@ -1782,7 +1963,7 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
@@ -1801,13 +1982,21 @@
         <v>35</v>
       </c>
       <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="C11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E11" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
@@ -1833,32 +2022,32 @@
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O12" s="10"/>
       <c r="P12" s="10"/>
@@ -1871,7 +2060,7 @@
       <c r="W12" s="11"/>
       <c r="X12" s="10"/>
       <c r="Y12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -1879,15 +2068,21 @@
         <v>37</v>
       </c>
       <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
+      <c r="C13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="E13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
@@ -1895,7 +2090,7 @@
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
       <c r="N13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
@@ -1908,7 +2103,7 @@
       <c r="W13" s="11"/>
       <c r="X13" s="10"/>
       <c r="Y13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -1917,35 +2112,37 @@
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="10"/>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="10"/>
@@ -1956,36 +2153,103 @@
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
       <c r="X14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y14" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25">
+      <c r="A15" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="Y14" s="10" t="s">
-        <v>27</v>
-      </c>
+      <c r="G15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
+      <c r="Y15" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:Y1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:Y14">
+  <conditionalFormatting sqref="W15:Y15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C14">
+  <conditionalFormatting sqref="W15:Y15">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W15:Y15">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:V15">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:V15">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:V15">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B3:Y14">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C14">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:Y14">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1994,14 +2258,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2020,7 +2284,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2030,25 +2294,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -2060,7 +2324,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2071,14 +2335,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2097,7 +2361,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2129,7 +2393,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2140,14 +2404,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2166,7 +2430,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2176,55 +2440,55 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B11" s="10"/>
     </row>
@@ -2236,7 +2500,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2247,14 +2511,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2273,7 +2537,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2283,19 +2547,19 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="10"/>
     </row>
@@ -2307,7 +2571,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2318,14 +2582,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2344,7 +2608,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2354,18 +2618,18 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="2:2">
@@ -2377,39 +2641,39 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2420,14 +2684,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2446,7 +2710,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2456,40 +2720,40 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -2500,7 +2764,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2511,14 +2775,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2537,7 +2801,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2557,7 +2821,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2568,14 +2832,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2594,7 +2858,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2604,131 +2868,131 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="10"/>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B12" s="10"/>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="10"/>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B14" s="10"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B16" s="10"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B17" s="10"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B18" s="10"/>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" s="10"/>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B20" s="10"/>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B21" s="10"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22" s="10"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B23" s="10"/>
       <c r="D23" s="10"/>
@@ -2739,29 +3003,29 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2772,14 +3036,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2798,7 +3062,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2808,37 +3072,37 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="10"/>
     </row>
@@ -2850,7 +3114,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2861,14 +3125,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2887,7 +3151,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2897,25 +3161,25 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6" s="10"/>
     </row>
@@ -2927,7 +3191,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2938,14 +3202,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2964,7 +3228,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -2974,37 +3238,37 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" s="10"/>
     </row>
@@ -3016,7 +3280,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3027,14 +3291,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3053,7 +3317,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -3063,31 +3327,31 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B7" s="10"/>
     </row>
@@ -3099,7 +3363,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1769990795" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3110,14 +3374,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1769990795" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1769990795" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Added tests for pointer
</commit_message>
<xml_diff>
--- a/php-zigar/tests/test-matrix.xlsx
+++ b/php-zigar/tests/test-matrix.xlsx
@@ -25,17 +25,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1772143101" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1772143101" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1772143101" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1772143101"/>
+      <pm:revision xmlns:pm="smNativeData" day="1773083893" val="1230" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1773083893" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1773083893" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1773083893"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="107">
   <si>
     <t>Context</t>
   </si>
@@ -385,7 +385,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1773083893" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -400,7 +400,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1773083893" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -415,7 +415,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1773083893" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -431,7 +431,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1772143101" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1773083893" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -453,7 +453,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -464,7 +464,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -475,7 +475,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -486,7 +486,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -497,7 +497,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -508,7 +508,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -519,7 +519,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -541,7 +541,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
+          <pm:border xmlns:pm="smNativeData" id="1773083893"/>
         </ext>
       </extLst>
     </border>
@@ -560,7 +560,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101">
+          <pm:border xmlns:pm="smNativeData" id="1773083893">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -582,7 +582,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101">
+          <pm:border xmlns:pm="smNativeData" id="1773083893">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -606,7 +606,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101">
+          <pm:border xmlns:pm="smNativeData" id="1773083893">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -630,7 +630,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101">
+          <pm:border xmlns:pm="smNativeData" id="1773083893">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -654,7 +654,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
+          <pm:border xmlns:pm="smNativeData" id="1773083893"/>
         </ext>
       </extLst>
     </border>
@@ -673,7 +673,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
+          <pm:border xmlns:pm="smNativeData" id="1773083893"/>
         </ext>
       </extLst>
     </border>
@@ -692,7 +692,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1772143101"/>
+          <pm:border xmlns:pm="smNativeData" id="1773083893"/>
         </ext>
       </extLst>
     </border>
@@ -742,13 +742,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="21">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -761,7 +761,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -772,7 +772,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -785,7 +785,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -796,7 +796,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -809,7 +809,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -820,7 +820,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -833,7 +833,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -844,7 +844,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -857,7 +857,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -868,7 +868,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -881,7 +881,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -892,7 +892,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -905,7 +905,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -916,7 +916,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -929,7 +929,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -940,7 +940,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -953,7 +953,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -964,7 +964,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -977,7 +977,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -988,7 +988,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1001,7 +1001,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1012,7 +1012,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1025,7 +1025,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1036,7 +1036,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1049,7 +1049,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1060,7 +1060,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1073,7 +1073,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1084,7 +1084,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1097,7 +1097,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1108,7 +1108,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1121,7 +1121,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1132,7 +1132,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1145,7 +1145,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1156,7 +1156,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1169,7 +1169,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1180,7 +1180,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1772143101" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1193,7 +1193,55 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1772143101" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1773083893" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1773083893" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1203,10 +1251,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1772143101" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1773083893" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1772143101" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1773083893" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -1615,7 +1663,9 @@
       <c r="A3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C3" s="10" t="s">
         <v>26</v>
       </c>
@@ -1631,9 +1681,15 @@
       <c r="G3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
+      <c r="H3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="K3" s="10" t="s">
         <v>26</v>
       </c>
@@ -1647,26 +1703,40 @@
         <v>26</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="P3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
+      <c r="U3" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
-      <c r="X3" s="10"/>
+      <c r="X3" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y3" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C4" s="10" t="s">
         <v>26</v>
       </c>
@@ -1682,31 +1752,51 @@
       <c r="G4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
+      <c r="H4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="K4" s="10" t="s">
         <v>26</v>
       </c>
       <c r="L4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="10"/>
+      <c r="M4" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="N4" s="10" t="s">
         <v>26</v>
       </c>
       <c r="O4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
+      <c r="P4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
+      <c r="U4" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
-      <c r="X4" s="10"/>
+      <c r="X4" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y4" s="10" t="s">
         <v>26</v>
       </c>
@@ -1715,7 +1805,9 @@
       <c r="A5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C5" s="10" t="s">
         <v>26</v>
       </c>
@@ -1723,7 +1815,7 @@
         <v>26</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>26</v>
@@ -1731,31 +1823,51 @@
       <c r="G5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
+      <c r="H5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="K5" s="10" t="s">
         <v>26</v>
       </c>
       <c r="L5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="10"/>
+      <c r="M5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="N5" s="10" t="s">
         <v>26</v>
       </c>
       <c r="O5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="10"/>
+      <c r="P5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S5" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T5" s="10"/>
-      <c r="U5" s="10"/>
+      <c r="U5" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
-      <c r="X5" s="10"/>
+      <c r="X5" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y5" s="10" t="s">
         <v>26</v>
       </c>
@@ -1764,7 +1876,9 @@
       <c r="A6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C6" s="10" t="s">
         <v>26</v>
       </c>
@@ -1778,38 +1892,64 @@
         <v>26</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="L6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M6" s="10"/>
+      <c r="M6" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="N6" s="10" t="s">
         <v>27</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S6" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T6" s="10"/>
-      <c r="U6" s="10"/>
+      <c r="U6" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V6" s="11"/>
       <c r="W6" s="11"/>
-      <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
+      <c r="X6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y6" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C7" s="10" t="s">
         <v>26</v>
       </c>
@@ -1825,32 +1965,62 @@
       <c r="G7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
+      <c r="H7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T7" s="10"/>
-      <c r="U7" s="10"/>
+      <c r="U7" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
-      <c r="X7" s="10"/>
+      <c r="X7" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C8" s="10" t="s">
         <v>26</v>
       </c>
@@ -1866,9 +2036,15 @@
       <c r="G8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
+      <c r="H8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="K8" s="10" t="s">
         <v>26</v>
       </c>
@@ -1884,15 +2060,29 @@
       <c r="O8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10"/>
+      <c r="P8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="T8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="U8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
-      <c r="X8" s="10"/>
+      <c r="X8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="Y8" s="10" t="s">
         <v>26</v>
       </c>
@@ -1901,7 +2091,9 @@
       <c r="A9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C9" s="10" t="s">
         <v>26</v>
       </c>
@@ -1917,30 +2109,62 @@
       <c r="G9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
+      <c r="H9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S9" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T9" s="10"/>
-      <c r="U9" s="10"/>
+      <c r="U9" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
-      <c r="X9" s="10"/>
-      <c r="Y9" s="10"/>
+      <c r="X9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y9" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C10" s="10" t="s">
         <v>26</v>
       </c>
@@ -1956,32 +2180,64 @@
       <c r="G10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
+      <c r="H10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="N10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="10"/>
+      <c r="O10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="T10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V10" s="11"/>
       <c r="W10" s="11"/>
-      <c r="X10" s="10"/>
-      <c r="Y10" s="10"/>
+      <c r="X10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y10" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C11" s="10" t="s">
         <v>26</v>
       </c>
@@ -1997,30 +2253,62 @@
       <c r="G11" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
-      <c r="S11" s="10"/>
+      <c r="H11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S11" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T11" s="10"/>
-      <c r="U11" s="10"/>
+      <c r="U11" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V11" s="11"/>
       <c r="W11" s="11"/>
-      <c r="X11" s="10"/>
-      <c r="Y11" s="10"/>
+      <c r="X11" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y11" s="10" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="12" spans="1:25">
       <c r="A12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="10"/>
+      <c r="B12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C12" s="10" t="s">
         <v>26</v>
       </c>
@@ -2036,29 +2324,51 @@
       <c r="G12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
+      <c r="H12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="K12" s="10" t="s">
         <v>26</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M12" s="10"/>
+      <c r="M12" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="N12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
+      <c r="O12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S12" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
+      <c r="U12" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V12" s="11"/>
       <c r="W12" s="11"/>
-      <c r="X12" s="10"/>
+      <c r="X12" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y12" s="10" t="s">
         <v>26</v>
       </c>
@@ -2067,7 +2377,9 @@
       <c r="A13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C13" s="10" t="s">
         <v>26</v>
       </c>
@@ -2083,25 +2395,51 @@
       <c r="G13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
+      <c r="H13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="N13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="10"/>
-      <c r="S13" s="10"/>
+      <c r="O13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="T13" s="10"/>
-      <c r="U13" s="10"/>
+      <c r="U13" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V13" s="11"/>
       <c r="W13" s="11"/>
-      <c r="X13" s="10"/>
+      <c r="X13" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="Y13" s="10" t="s">
         <v>26</v>
       </c>
@@ -2110,7 +2448,9 @@
       <c r="A14" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="10"/>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="C14" s="10" t="s">
         <v>26</v>
       </c>
@@ -2124,11 +2464,17 @@
         <v>26</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
+        <v>26</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="K14" s="10" t="s">
         <v>26</v>
       </c>
@@ -2144,12 +2490,24 @@
       <c r="O14" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
+      <c r="P14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="T14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
       <c r="X14" s="10" t="s">
@@ -2163,14 +2521,18 @@
       <c r="A15" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C15" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="F15" s="10" t="s">
         <v>27</v>
       </c>
@@ -2178,21 +2540,35 @@
         <v>26</v>
       </c>
       <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
+      <c r="I15" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
+      <c r="K15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
+      <c r="N15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
+      <c r="R15" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="S15" s="10"/>
       <c r="T15" s="10"/>
-      <c r="U15" s="10"/>
-      <c r="V15" s="10"/>
-      <c r="W15" s="10"/>
+      <c r="U15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="10"/>
     </row>
@@ -2201,55 +2577,65 @@
     <mergeCell ref="B1:Y1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <conditionalFormatting sqref="W15:Y15">
+  <conditionalFormatting sqref="V15:W15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W15:Y15">
+  <conditionalFormatting sqref="V15:W15">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X15:Y15">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W15:Y15">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>N</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:V15">
+  <conditionalFormatting sqref="X15:Y15">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:V15">
+  <conditionalFormatting sqref="X15:Y15">
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>N</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:U15">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:V15">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+  <conditionalFormatting sqref="B15:U15">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:U15">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:Y14">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C14">
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:Y14">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2258,14 +2644,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2324,7 +2710,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2335,14 +2721,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2393,7 +2779,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2404,14 +2790,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2500,7 +2886,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2511,14 +2897,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2571,7 +2957,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2582,14 +2968,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2641,39 +3027,39 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6">
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="14" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2684,14 +3070,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2764,7 +3150,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2775,14 +3161,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2821,7 +3207,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2832,14 +3218,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3003,29 +3389,29 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D23">
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B23">
-    <cfRule type="cellIs" dxfId="18" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="4" operator="equal">
       <formula>N</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3036,14 +3422,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3114,7 +3500,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3125,14 +3511,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3191,7 +3577,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3202,14 +3588,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3280,7 +3666,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3291,14 +3677,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3363,7 +3749,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1772143101" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1773083893" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3374,14 +3760,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1772143101" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1773083893" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1772143101" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1773083893" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>